<commit_message>
actualizados costos energia, detenciones y asignaciones
</commit_message>
<xml_diff>
--- a/data/Escenarios_DET/carga_on_board_costo_fijo/simple_time_series.xlsx
+++ b/data/Escenarios_DET/carga_on_board_costo_fijo/simple_time_series.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="MarginalCost" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Shifts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="NodeAssignment" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="StationAssignment" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ExtractionGoal" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MarginalCost" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shifts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NodeAssignment" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StationAssignment" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExtractionGoal" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25035,7 +25035,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LH518B_2</t>
+          <t>LH518B_1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -25060,7 +25060,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>LH518B_2</t>
+          <t>LH518B_1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -25085,7 +25085,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>LH518B_2</t>
+          <t>LH518B_1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -25110,7 +25110,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>LH518B_2</t>
+          <t>LH518B_1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -25135,7 +25135,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LH518B_2</t>
+          <t>LH518B_1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -25160,7 +25160,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LH518B_2</t>
+          <t>LH518B_1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -25510,7 +25510,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -25535,7 +25535,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -25560,7 +25560,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -25585,7 +25585,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -25610,7 +25610,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -25635,7 +25635,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -25660,7 +25660,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -25685,7 +25685,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -25710,7 +25710,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -25735,7 +25735,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -25760,7 +25760,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -25785,7 +25785,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -25810,7 +25810,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>LH518B_3</t>
+          <t>LH518B_2</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -26110,7 +26110,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -26135,7 +26135,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -26160,7 +26160,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -26185,7 +26185,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -26210,7 +26210,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -26235,7 +26235,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -26260,7 +26260,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -26285,7 +26285,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -26310,7 +26310,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -26335,7 +26335,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -26360,7 +26360,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -26385,7 +26385,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -26410,7 +26410,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -26435,7 +26435,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -26460,7 +26460,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -26485,7 +26485,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>LH518B_4</t>
+          <t>LH518B_3</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -26710,7 +26710,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -26735,7 +26735,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -26760,7 +26760,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -26785,7 +26785,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -26810,7 +26810,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -26835,7 +26835,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -26860,7 +26860,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -26885,7 +26885,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -26910,7 +26910,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -26935,7 +26935,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -26960,7 +26960,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -26985,7 +26985,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -27010,7 +27010,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -27035,7 +27035,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -27060,7 +27060,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -27085,7 +27085,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -27110,7 +27110,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -27135,7 +27135,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -27160,7 +27160,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -27185,7 +27185,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>LH518B_5</t>
+          <t>LH518B_4</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -27310,7 +27310,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -27335,7 +27335,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -27360,7 +27360,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -27385,7 +27385,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -27410,7 +27410,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -27435,7 +27435,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -27460,7 +27460,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -27485,7 +27485,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -27510,7 +27510,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -27535,7 +27535,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -27560,7 +27560,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -27585,7 +27585,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -27610,7 +27610,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -27635,7 +27635,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -27660,7 +27660,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -27685,7 +27685,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -27710,7 +27710,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -27735,7 +27735,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -27760,7 +27760,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -27785,7 +27785,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -27810,7 +27810,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -27835,7 +27835,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -27860,7 +27860,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>LH518B_6</t>
+          <t>LH518B_5</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -27885,7 +27885,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -27910,7 +27910,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -27935,7 +27935,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -27960,7 +27960,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -27985,7 +27985,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -28010,7 +28010,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -28035,7 +28035,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -28060,7 +28060,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -28085,7 +28085,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -28110,7 +28110,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -28135,7 +28135,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -28160,7 +28160,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -28185,7 +28185,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -28210,7 +28210,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -28235,7 +28235,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -28260,7 +28260,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -28285,7 +28285,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -28310,7 +28310,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -28335,7 +28335,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -28360,7 +28360,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -28385,7 +28385,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -28410,7 +28410,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -28435,7 +28435,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -28460,7 +28460,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>LH518B_7</t>
+          <t>LH518B_6</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -28535,7 +28535,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -28560,7 +28560,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -28585,7 +28585,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -28610,7 +28610,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -28635,7 +28635,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -28660,7 +28660,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -28685,7 +28685,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -28710,7 +28710,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -28735,7 +28735,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -28760,7 +28760,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -28785,7 +28785,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -28810,7 +28810,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -28835,7 +28835,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -28860,7 +28860,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -28885,7 +28885,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -28910,7 +28910,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -28935,7 +28935,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -28960,7 +28960,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>LH518B_8</t>
+          <t>LH518B_7</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -29235,7 +29235,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>LH518B_9</t>
+          <t>LH518B_8</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -29260,7 +29260,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>LH518B_9</t>
+          <t>LH518B_8</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
@@ -29285,7 +29285,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>LH518B_9</t>
+          <t>LH518B_8</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -29310,7 +29310,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>LH518B_9</t>
+          <t>LH518B_8</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -29335,7 +29335,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>LH518B_9</t>
+          <t>LH518B_8</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -29360,7 +29360,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>LH518B_9</t>
+          <t>LH518B_8</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">

</xml_diff>